<commit_message>
Changes to excels to add technologies and two demands + changes to ReadMe
</commit_message>
<xml_diff>
--- a/Group Assignment MfT/input_databases/default/technologies.xlsx
+++ b/Group Assignment MfT/input_databases/default/technologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling _for_Transitions/P06_STUDENT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling_for_transitions_Group/Group Assignment MfT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66C8799B-78A8-6642-B161-1F9CC1867E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEAD918F-2CF4-A748-8E08-59B83AD8A7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3560" yWindow="600" windowWidth="13660" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="105">
   <si>
     <t>Technology</t>
   </si>
@@ -266,9 +266,6 @@
     <t>Gas boiler to generate space and water heating</t>
   </si>
   <si>
-    <t>Residential heat</t>
-  </si>
-  <si>
     <t>Residential heat pump</t>
   </si>
   <si>
@@ -351,6 +348,15 @@
   </si>
   <si>
     <t>Generic industrial high temperature process running on fossil energy - existing base</t>
+  </si>
+  <si>
+    <t>Residential heat low</t>
+  </si>
+  <si>
+    <t>Residential heat high</t>
+  </si>
+  <si>
+    <t>Subsidy</t>
   </si>
 </sst>
 </file>
@@ -685,7 +691,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2AEF3F7-9EA9-4235-9872-78FDC34EDD32}">
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -1496,7 +1502,7 @@
         <v>9</v>
       </c>
       <c r="E75" t="s">
-        <v>74</v>
+        <v>102</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1514,796 +1520,824 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+      <c r="B77" t="s">
+        <v>66</v>
+      </c>
+      <c r="C77" t="s">
+        <v>32</v>
+      </c>
+      <c r="D77" t="s">
+        <v>9</v>
+      </c>
+      <c r="E77" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>74</v>
+      </c>
+      <c r="B78" t="s">
+        <v>49</v>
+      </c>
+      <c r="E78" t="s">
         <v>75</v>
-      </c>
-      <c r="B77" t="s">
-        <v>49</v>
-      </c>
-      <c r="E77" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B78" t="s">
-        <v>16</v>
-      </c>
-      <c r="E78" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E79" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
-        <v>28</v>
-      </c>
-      <c r="C80" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E80" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
+        <v>28</v>
+      </c>
+      <c r="C81" t="s">
+        <v>29</v>
+      </c>
+      <c r="E81" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B82" t="s">
         <v>31</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C82" t="s">
         <v>32</v>
       </c>
-      <c r="D81" t="s">
-        <v>9</v>
-      </c>
-      <c r="E81" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+      <c r="D82" t="s">
+        <v>9</v>
+      </c>
+      <c r="E82" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>76</v>
+      </c>
+      <c r="B83" t="s">
+        <v>49</v>
+      </c>
+      <c r="E83" t="s">
         <v>77</v>
-      </c>
-      <c r="B82" t="s">
-        <v>49</v>
-      </c>
-      <c r="E82" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B83" t="s">
-        <v>16</v>
-      </c>
-      <c r="E83" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E84" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
-        <v>28</v>
-      </c>
-      <c r="C85" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E85" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B86" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C86" t="s">
-        <v>32</v>
-      </c>
-      <c r="D86" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E86" t="s">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
+        <v>31</v>
+      </c>
+      <c r="C87" t="s">
+        <v>32</v>
+      </c>
+      <c r="D87" t="s">
+        <v>9</v>
+      </c>
+      <c r="E87" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B88" t="s">
         <v>46</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C88" t="s">
         <v>47</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D88" t="s">
         <v>44</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E88" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>80</v>
+      </c>
+      <c r="B89" t="s">
+        <v>49</v>
+      </c>
+      <c r="E89" t="s">
         <v>81</v>
-      </c>
-      <c r="B88" t="s">
-        <v>49</v>
-      </c>
-      <c r="E88" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B89" t="s">
-        <v>16</v>
-      </c>
-      <c r="E89" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E90" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
-        <v>28</v>
-      </c>
-      <c r="C91" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E91" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B92" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C92" t="s">
-        <v>32</v>
-      </c>
-      <c r="D92" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E92" t="s">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C93" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="D93" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="E93" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C94" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="D94" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="E94" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
+        <v>66</v>
+      </c>
+      <c r="C95" t="s">
+        <v>67</v>
+      </c>
+      <c r="D95" t="s">
+        <v>68</v>
+      </c>
+      <c r="E95" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B96" t="s">
         <v>52</v>
       </c>
-      <c r="E95">
+      <c r="E96">
         <v>2030</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>82</v>
+      </c>
+      <c r="B97" t="s">
+        <v>49</v>
+      </c>
+      <c r="E97" t="s">
         <v>83</v>
-      </c>
-      <c r="B96" t="s">
-        <v>49</v>
-      </c>
-      <c r="E96" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B97" t="s">
-        <v>16</v>
-      </c>
-      <c r="E97" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E98" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
-        <v>28</v>
-      </c>
-      <c r="C99" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E99" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
+        <v>28</v>
+      </c>
+      <c r="C100" t="s">
+        <v>29</v>
+      </c>
+      <c r="E100" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B101" t="s">
         <v>31</v>
       </c>
-      <c r="C100" t="s">
+      <c r="C101" t="s">
         <v>32</v>
       </c>
-      <c r="D100" t="s">
-        <v>9</v>
-      </c>
-      <c r="E100" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+      <c r="D101" t="s">
+        <v>9</v>
+      </c>
+      <c r="E101" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>84</v>
+      </c>
+      <c r="B102" t="s">
+        <v>49</v>
+      </c>
+      <c r="E102" t="s">
         <v>85</v>
-      </c>
-      <c r="B101" t="s">
-        <v>49</v>
-      </c>
-      <c r="E101" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B102" t="s">
-        <v>16</v>
-      </c>
-      <c r="E102" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E103" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B104" t="s">
-        <v>28</v>
-      </c>
-      <c r="C104" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E104" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C105" t="s">
-        <v>32</v>
-      </c>
-      <c r="D105" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E105" t="s">
-        <v>87</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
+        <v>31</v>
+      </c>
+      <c r="C106" t="s">
+        <v>32</v>
+      </c>
+      <c r="D106" t="s">
+        <v>9</v>
+      </c>
+      <c r="E106" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B107" t="s">
         <v>46</v>
       </c>
-      <c r="C106" t="s">
+      <c r="C107" t="s">
         <v>47</v>
       </c>
-      <c r="D106" t="s">
+      <c r="D107" t="s">
         <v>44</v>
       </c>
-      <c r="E106" t="s">
+      <c r="E107" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>87</v>
+      </c>
+      <c r="B108" t="s">
+        <v>49</v>
+      </c>
+      <c r="E108" t="s">
         <v>88</v>
-      </c>
-      <c r="B107" t="s">
-        <v>49</v>
-      </c>
-      <c r="E107" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B108" t="s">
-        <v>16</v>
-      </c>
-      <c r="E108" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E109" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
-        <v>28</v>
-      </c>
-      <c r="C110" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E110" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C111" t="s">
-        <v>32</v>
-      </c>
-      <c r="D111" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E111" t="s">
-        <v>87</v>
+        <v>30</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C112" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="D112" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="E112" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C113" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="D113" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="E113" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
+        <v>66</v>
+      </c>
+      <c r="C114" t="s">
+        <v>67</v>
+      </c>
+      <c r="D114" t="s">
+        <v>68</v>
+      </c>
+      <c r="E114" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B115" t="s">
         <v>52</v>
       </c>
-      <c r="E114">
+      <c r="E115">
         <v>2030</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>95</v>
-      </c>
-      <c r="B115" t="s">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>94</v>
+      </c>
+      <c r="B116" t="s">
         <v>49</v>
       </c>
-      <c r="E115" t="s">
+      <c r="E116" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B116" t="s">
-        <v>16</v>
-      </c>
-      <c r="E116" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E117" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>28</v>
-      </c>
-      <c r="C118" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E118" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
+        <v>28</v>
+      </c>
+      <c r="C119" t="s">
+        <v>29</v>
+      </c>
+      <c r="E119" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B120" t="s">
         <v>31</v>
       </c>
-      <c r="C119" t="s">
+      <c r="C120" t="s">
         <v>32</v>
       </c>
-      <c r="D119" t="s">
-        <v>9</v>
-      </c>
-      <c r="E119" t="s">
+      <c r="D120" t="s">
+        <v>9</v>
+      </c>
+      <c r="E120" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
-        <v>97</v>
-      </c>
-      <c r="B120" t="s">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>96</v>
+      </c>
+      <c r="B121" t="s">
         <v>49</v>
       </c>
-      <c r="E120" t="s">
+      <c r="E121" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B121" t="s">
-        <v>16</v>
-      </c>
-      <c r="E121" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E122" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
-        <v>28</v>
-      </c>
-      <c r="C123" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E123" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C124" t="s">
-        <v>32</v>
-      </c>
-      <c r="D124" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E124" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
+        <v>31</v>
+      </c>
+      <c r="C125" t="s">
+        <v>32</v>
+      </c>
+      <c r="D125" t="s">
+        <v>9</v>
+      </c>
+      <c r="E125" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B126" t="s">
         <v>46</v>
       </c>
-      <c r="C125" t="s">
+      <c r="C126" t="s">
         <v>47</v>
       </c>
-      <c r="D125" t="s">
+      <c r="D126" t="s">
         <v>44</v>
       </c>
-      <c r="E125" t="s">
+      <c r="E126" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
-        <v>94</v>
-      </c>
-      <c r="B126" t="s">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>93</v>
+      </c>
+      <c r="B127" t="s">
         <v>49</v>
       </c>
-      <c r="E126" t="s">
+      <c r="E127" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B127" t="s">
-        <v>16</v>
-      </c>
-      <c r="E127" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E128" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
-        <v>28</v>
-      </c>
-      <c r="C129" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E129" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C130" t="s">
-        <v>32</v>
-      </c>
-      <c r="D130" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E130" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
+        <v>31</v>
+      </c>
+      <c r="C131" t="s">
+        <v>32</v>
+      </c>
+      <c r="D131" t="s">
+        <v>9</v>
+      </c>
+      <c r="E131" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B132" t="s">
         <v>46</v>
       </c>
-      <c r="C131" t="s">
+      <c r="C132" t="s">
         <v>47</v>
       </c>
-      <c r="D131" t="s">
+      <c r="D132" t="s">
         <v>44</v>
       </c>
-      <c r="E131" t="s">
+      <c r="E132" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
-        <v>100</v>
-      </c>
-      <c r="B132" t="s">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
+        <v>99</v>
+      </c>
+      <c r="B133" t="s">
         <v>49</v>
       </c>
-      <c r="E132" t="s">
+      <c r="E133" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B133" t="s">
-        <v>16</v>
-      </c>
-      <c r="E133" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E134" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
-        <v>28</v>
-      </c>
-      <c r="C135" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E135" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C136" t="s">
-        <v>32</v>
-      </c>
-      <c r="D136" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E136" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
+        <v>31</v>
+      </c>
+      <c r="C137" t="s">
+        <v>32</v>
+      </c>
+      <c r="D137" t="s">
+        <v>9</v>
+      </c>
+      <c r="E137" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B138" t="s">
         <v>46</v>
       </c>
-      <c r="C137" t="s">
+      <c r="C138" t="s">
         <v>47</v>
       </c>
-      <c r="D137" t="s">
+      <c r="D138" t="s">
         <v>44</v>
       </c>
-      <c r="E137" t="s">
+      <c r="E138" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
-        <v>98</v>
-      </c>
-      <c r="B138" t="s">
-        <v>49</v>
-      </c>
-      <c r="E138" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
-        <v>16</v>
+        <v>66</v>
+      </c>
+      <c r="C139" t="s">
+        <v>32</v>
+      </c>
+      <c r="D139" t="s">
+        <v>9</v>
       </c>
       <c r="E139" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>97</v>
+      </c>
       <c r="B140" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="E140" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
-        <v>28</v>
-      </c>
-      <c r="C141" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E141" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
-        <v>31</v>
-      </c>
-      <c r="C142" t="s">
-        <v>32</v>
-      </c>
-      <c r="D142" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E142" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
+        <v>28</v>
+      </c>
+      <c r="C143" t="s">
+        <v>29</v>
+      </c>
+      <c r="E143" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B144" t="s">
+        <v>31</v>
+      </c>
+      <c r="C144" t="s">
+        <v>32</v>
+      </c>
+      <c r="D144" t="s">
+        <v>9</v>
+      </c>
+      <c r="E144" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B145" t="s">
         <v>46</v>
       </c>
-      <c r="C143" t="s">
+      <c r="C145" t="s">
         <v>47</v>
       </c>
-      <c r="D143" t="s">
+      <c r="D145" t="s">
         <v>44</v>
       </c>
-      <c r="E143" t="s">
+      <c r="E145" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>99</v>
-      </c>
-      <c r="B144" t="s">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>98</v>
+      </c>
+      <c r="B146" t="s">
         <v>49</v>
       </c>
-      <c r="E144" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="145" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B145" t="s">
+      <c r="E146" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B147" t="s">
         <v>16</v>
       </c>
-      <c r="E145" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="146" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B146" t="s">
+      <c r="E147" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B148" t="s">
         <v>24</v>
       </c>
-      <c r="E146" t="s">
+      <c r="E148" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B147" t="s">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B149" t="s">
         <v>28</v>
       </c>
-      <c r="C147" t="s">
+      <c r="C149" t="s">
         <v>29</v>
       </c>
-      <c r="E147" t="s">
+      <c r="E149" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="148" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B148" t="s">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B150" t="s">
         <v>31</v>
       </c>
-      <c r="C148" t="s">
+      <c r="C150" t="s">
         <v>32</v>
       </c>
-      <c r="D148" t="s">
-        <v>9</v>
-      </c>
-      <c r="E148" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="149" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B149" t="s">
+      <c r="D150" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B151" t="s">
         <v>46</v>
       </c>
-      <c r="C149" t="s">
+      <c r="C151" t="s">
         <v>47</v>
       </c>
-      <c r="D149" t="s">
+      <c r="D151" t="s">
         <v>44</v>
       </c>
-      <c r="E149" t="s">
+      <c r="E151" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2316,7 +2350,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -3455,7 +3489,7 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B74" t="s">
         <v>6</v>
@@ -3464,542 +3498,542 @@
         <v>21</v>
       </c>
       <c r="D74">
+        <v>2200</v>
+      </c>
+      <c r="E74">
         <v>2000</v>
-      </c>
-      <c r="E74">
-        <v>1500</v>
-      </c>
-      <c r="G74">
-        <v>500</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
       <c r="C75" t="s">
         <v>21</v>
       </c>
       <c r="D75">
-        <f>D74*0.05</f>
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E75">
-        <f>E74*0.05</f>
-        <v>75</v>
-      </c>
-      <c r="G75">
-        <f>G74*0.05</f>
-        <v>25</v>
+        <v>200</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C76" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D76">
+        <f>D74*0.05</f>
+        <v>110</v>
+      </c>
+      <c r="E76">
+        <f>E75*0.05</f>
+        <v>10</v>
+      </c>
+      <c r="G76">
+        <f>G75*0.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C77" t="s">
+        <v>22</v>
       </c>
       <c r="D77">
-        <v>3</v>
-      </c>
-      <c r="E77">
-        <v>4</v>
-      </c>
-      <c r="G77">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D78">
+        <v>3</v>
+      </c>
+      <c r="E78">
+        <v>4</v>
+      </c>
+      <c r="G78">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B79" t="s">
         <v>10</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C79" t="s">
         <v>11</v>
       </c>
-      <c r="D78">
+      <c r="D79">
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>77</v>
-      </c>
-      <c r="B79" t="s">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>76</v>
+      </c>
+      <c r="B80" t="s">
         <v>6</v>
-      </c>
-      <c r="C79" t="s">
-        <v>21</v>
-      </c>
-      <c r="D79">
-        <v>450</v>
-      </c>
-      <c r="G79">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B80" t="s">
-        <v>7</v>
       </c>
       <c r="C80" t="s">
         <v>21</v>
       </c>
       <c r="D80">
-        <f>D79*0.05</f>
-        <v>22.5</v>
+        <v>450</v>
       </c>
       <c r="G80">
-        <f>G79*0.05</f>
-        <v>15</v>
+        <v>300</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C81" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D81">
-        <v>0.2</v>
+        <f>D80*0.05</f>
+        <v>22.5</v>
       </c>
       <c r="G81">
-        <v>0.2</v>
+        <f>G80*0.05</f>
+        <v>15</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C82" t="s">
+        <v>22</v>
       </c>
       <c r="D82">
-        <v>0.85</v>
+        <v>0.2</v>
       </c>
       <c r="G82">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
-        <v>10</v>
-      </c>
-      <c r="C83" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D83">
-        <v>20</v>
+        <v>0.85</v>
       </c>
       <c r="G83">
-        <v>20</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
+        <v>10</v>
+      </c>
+      <c r="C84" t="s">
+        <v>11</v>
+      </c>
+      <c r="D84">
+        <v>20</v>
+      </c>
+      <c r="G84">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B85" t="s">
         <v>44</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C85" t="s">
         <v>45</v>
       </c>
-      <c r="D84">
+      <c r="D85">
         <v>0.2</v>
       </c>
-      <c r="G84">
+      <c r="G85">
         <v>0.2</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>81</v>
-      </c>
-      <c r="B85" t="s">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>80</v>
+      </c>
+      <c r="B86" t="s">
         <v>6</v>
-      </c>
-      <c r="C85" t="s">
-        <v>21</v>
-      </c>
-      <c r="D85">
-        <f>D79*2</f>
-        <v>900</v>
-      </c>
-      <c r="G85">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B86" t="s">
-        <v>7</v>
       </c>
       <c r="C86" t="s">
         <v>21</v>
       </c>
       <c r="D86">
-        <f>D85*0.05</f>
-        <v>45</v>
+        <f>D80*2</f>
+        <v>900</v>
       </c>
       <c r="G86">
-        <f>G85*0.05</f>
-        <v>25</v>
+        <v>500</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B87" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C87" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D87">
-        <v>0.4</v>
+        <f>D86*0.05</f>
+        <v>45</v>
       </c>
       <c r="G87">
-        <v>0.3</v>
+        <f>G86*0.05</f>
+        <v>25</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B88" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C88" t="s">
+        <v>22</v>
       </c>
       <c r="D88">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G88">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B89" t="s">
-        <v>10</v>
-      </c>
-      <c r="C89" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D89">
-        <v>20</v>
+        <v>0.8</v>
       </c>
       <c r="G89">
-        <v>20</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
+        <v>10</v>
+      </c>
+      <c r="C90" t="s">
+        <v>11</v>
+      </c>
+      <c r="D90">
+        <v>20</v>
+      </c>
+      <c r="G90">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B91" t="s">
         <v>44</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C91" t="s">
         <v>45</v>
       </c>
-      <c r="D90">
+      <c r="D91">
         <f>0.2*0.15</f>
         <v>0.03</v>
       </c>
-      <c r="G90">
+      <c r="G91">
         <f>0.2*0.1</f>
         <v>2.0000000000000004E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B91" t="s">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B92" t="s">
         <v>68</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C92" t="s">
         <v>45</v>
       </c>
-      <c r="D91">
+      <c r="D92">
         <f>0.2*0.85</f>
         <v>0.17</v>
       </c>
-      <c r="G91">
+      <c r="G92">
         <f>0.2*0.9</f>
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>83</v>
-      </c>
-      <c r="B92" t="s">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>82</v>
+      </c>
+      <c r="B93" t="s">
         <v>6</v>
-      </c>
-      <c r="C92" t="s">
-        <v>21</v>
-      </c>
-      <c r="D92">
-        <v>350</v>
-      </c>
-      <c r="G92">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B93" t="s">
-        <v>7</v>
       </c>
       <c r="C93" t="s">
         <v>21</v>
       </c>
       <c r="D93">
-        <f>D92*0.05</f>
-        <v>17.5</v>
+        <v>350</v>
       </c>
       <c r="G93">
-        <f>G92*0.05</f>
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C94" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D94">
-        <v>0.2</v>
+        <f>D93*0.05</f>
+        <v>17.5</v>
       </c>
       <c r="G94">
-        <v>0.2</v>
+        <f>G93*0.05</f>
+        <v>5</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C95" t="s">
+        <v>22</v>
       </c>
       <c r="D95">
-        <v>0.95</v>
+        <v>0.2</v>
       </c>
       <c r="G95">
-        <v>0.99</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
+        <v>9</v>
+      </c>
+      <c r="D96">
+        <v>0.95</v>
+      </c>
+      <c r="G96">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B97" t="s">
         <v>10</v>
       </c>
-      <c r="C96" t="s">
+      <c r="C97" t="s">
         <v>11</v>
       </c>
-      <c r="D96">
+      <c r="D97">
         <v>15</v>
       </c>
-      <c r="G96">
+      <c r="G97">
         <v>20</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>85</v>
-      </c>
-      <c r="B97" t="s">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>84</v>
+      </c>
+      <c r="B98" t="s">
         <v>6</v>
-      </c>
-      <c r="C97" t="s">
-        <v>21</v>
-      </c>
-      <c r="D97">
-        <v>900</v>
-      </c>
-      <c r="G97">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B98" t="s">
-        <v>7</v>
       </c>
       <c r="C98" t="s">
         <v>21</v>
       </c>
       <c r="D98">
-        <f>D97*0.05</f>
-        <v>45</v>
+        <v>900</v>
       </c>
       <c r="G98">
-        <f>G97*0.05</f>
-        <v>20</v>
+        <v>400</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C99" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D99">
-        <v>0.2</v>
+        <f>D98*0.05</f>
+        <v>45</v>
       </c>
       <c r="G99">
-        <v>0.2</v>
+        <f>G98*0.05</f>
+        <v>20</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C100" t="s">
+        <v>22</v>
       </c>
       <c r="D100">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G100">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
-        <v>10</v>
-      </c>
-      <c r="C101" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D101">
-        <v>20</v>
+        <v>0.6</v>
       </c>
       <c r="G101">
-        <v>20</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
+        <v>10</v>
+      </c>
+      <c r="C102" t="s">
+        <v>11</v>
+      </c>
+      <c r="D102">
+        <v>20</v>
+      </c>
+      <c r="G102">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B103" t="s">
         <v>44</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C103" t="s">
         <v>45</v>
       </c>
-      <c r="D102">
+      <c r="D103">
         <v>0.2</v>
       </c>
-      <c r="G102">
+      <c r="G103">
         <v>0.2</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>88</v>
-      </c>
-      <c r="B103" t="s">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>87</v>
+      </c>
+      <c r="B104" t="s">
         <v>6</v>
-      </c>
-      <c r="C103" t="s">
-        <v>21</v>
-      </c>
-      <c r="D103">
-        <f>D97*2</f>
-        <v>1800</v>
-      </c>
-      <c r="G103">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B104" t="s">
-        <v>7</v>
       </c>
       <c r="C104" t="s">
         <v>21</v>
       </c>
       <c r="D104">
-        <f>D103*0.05</f>
-        <v>90</v>
+        <f>D98*2</f>
+        <v>1800</v>
       </c>
       <c r="G104">
-        <f>G103*0.05</f>
-        <v>50</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B105" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C105" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D105">
-        <v>0.4</v>
+        <f>D104*0.05</f>
+        <v>90</v>
       </c>
       <c r="G105">
-        <v>0.3</v>
+        <f>G104*0.05</f>
+        <v>50</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C106" t="s">
+        <v>22</v>
       </c>
       <c r="D106">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G106">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
-        <v>10</v>
-      </c>
-      <c r="C107" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D107">
-        <v>20</v>
+        <v>0.5</v>
       </c>
       <c r="G107">
-        <v>20</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
+        <v>10</v>
+      </c>
+      <c r="C108" t="s">
+        <v>11</v>
+      </c>
+      <c r="D108">
+        <v>20</v>
+      </c>
+      <c r="G108">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B109" t="s">
         <v>44</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C109" t="s">
         <v>45</v>
       </c>
-      <c r="D108">
+      <c r="D109">
         <f>0.2*0.15</f>
         <v>0.03</v>
       </c>
-      <c r="G108">
+      <c r="G109">
         <f>0.2*0.1</f>
         <v>2.0000000000000004E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B109" t="s">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B110" t="s">
         <v>68</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C110" t="s">
         <v>45</v>
       </c>
-      <c r="D109">
+      <c r="D110">
         <f>0.2*0.85</f>
         <v>0.17</v>
       </c>
-      <c r="G109">
+      <c r="G110">
         <f>0.2*0.9</f>
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>95</v>
-      </c>
-      <c r="B110" t="s">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>94</v>
+      </c>
+      <c r="B111" t="s">
         <v>6</v>
-      </c>
-      <c r="C110" t="s">
-        <v>23</v>
-      </c>
-      <c r="D110">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B111" t="s">
-        <v>7</v>
       </c>
       <c r="C111" t="s">
         <v>23</v>
@@ -4010,10 +4044,10 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C112" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D112">
         <v>0</v>
@@ -4021,43 +4055,43 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C113" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D113">
-        <v>2.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
+        <v>9</v>
+      </c>
+      <c r="C114" t="s">
+        <v>20</v>
+      </c>
+      <c r="D114">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B115" t="s">
         <v>10</v>
       </c>
-      <c r="C114" t="s">
+      <c r="C115" t="s">
         <v>11</v>
       </c>
-      <c r="D114">
+      <c r="D115">
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>97</v>
-      </c>
-      <c r="B115" t="s">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>96</v>
+      </c>
+      <c r="B116" t="s">
         <v>6</v>
-      </c>
-      <c r="C115" t="s">
-        <v>23</v>
-      </c>
-      <c r="D115">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B116" t="s">
-        <v>7</v>
       </c>
       <c r="C116" t="s">
         <v>23</v>
@@ -4068,10 +4102,10 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C117" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D117">
         <v>0</v>
@@ -4079,299 +4113,310 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C118" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D118">
-        <v>2.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C119" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D119">
-        <v>4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
+        <v>10</v>
+      </c>
+      <c r="C120" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B121" t="s">
         <v>44</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C121" t="s">
         <v>45</v>
       </c>
-      <c r="D120">
+      <c r="D121">
         <v>0.25</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
-        <v>94</v>
-      </c>
-      <c r="B121" t="s">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>93</v>
+      </c>
+      <c r="B122" t="s">
         <v>6</v>
-      </c>
-      <c r="C121" t="s">
-        <v>21</v>
-      </c>
-      <c r="D121">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B122" t="s">
-        <v>7</v>
       </c>
       <c r="C122" t="s">
         <v>21</v>
       </c>
       <c r="D122">
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C123" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D123">
-        <v>0.2</v>
+        <v>48</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C124" t="s">
+        <v>22</v>
       </c>
       <c r="D124">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
-        <v>10</v>
-      </c>
-      <c r="C125" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D125">
-        <v>4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
+        <v>10</v>
+      </c>
+      <c r="C126" t="s">
+        <v>11</v>
+      </c>
+      <c r="D126">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B127" t="s">
         <v>44</v>
       </c>
-      <c r="C126" t="s">
+      <c r="C127" t="s">
         <v>45</v>
       </c>
-      <c r="D126">
+      <c r="D127">
         <v>0.2</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>100</v>
-      </c>
-      <c r="B127" t="s">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>99</v>
+      </c>
+      <c r="B128" t="s">
         <v>6</v>
-      </c>
-      <c r="C127" t="s">
-        <v>21</v>
-      </c>
-      <c r="D127">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B128" t="s">
-        <v>7</v>
       </c>
       <c r="C128" t="s">
         <v>21</v>
       </c>
       <c r="D128">
-        <f>D127*0.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C129" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D129">
+        <f>D128*0.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C130" t="s">
+        <v>22</v>
       </c>
       <c r="D130">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
-        <v>10</v>
-      </c>
-      <c r="C131" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D131">
-        <v>4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
+        <v>10</v>
+      </c>
+      <c r="C132" t="s">
+        <v>11</v>
+      </c>
+      <c r="D132">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B133" t="s">
         <v>44</v>
       </c>
-      <c r="C132" t="s">
+      <c r="C133" t="s">
         <v>45</v>
       </c>
-      <c r="D132">
+      <c r="D133">
         <v>0.2</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
-        <v>98</v>
-      </c>
-      <c r="B133" t="s">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
+        <v>97</v>
+      </c>
+      <c r="B134" t="s">
         <v>6</v>
-      </c>
-      <c r="C133" t="s">
-        <v>21</v>
-      </c>
-      <c r="D133">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B134" t="s">
-        <v>7</v>
       </c>
       <c r="C134" t="s">
         <v>21</v>
       </c>
       <c r="D134">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C135" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D135">
-        <v>0.1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C136" t="s">
+        <v>22</v>
       </c>
       <c r="D136">
-        <v>0.85</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
-        <v>10</v>
-      </c>
-      <c r="C137" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D137">
-        <v>4</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
+        <v>10</v>
+      </c>
+      <c r="C138" t="s">
+        <v>11</v>
+      </c>
+      <c r="D138">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B139" t="s">
         <v>44</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C139" t="s">
         <v>45</v>
       </c>
-      <c r="D138">
+      <c r="D139">
         <v>0.2</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
-        <v>99</v>
-      </c>
-      <c r="B139" t="s">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
+        <v>98</v>
+      </c>
+      <c r="B140" t="s">
         <v>6</v>
-      </c>
-      <c r="C139" t="s">
-        <v>21</v>
-      </c>
-      <c r="D139">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B140" t="s">
-        <v>7</v>
       </c>
       <c r="C140" t="s">
         <v>21</v>
       </c>
       <c r="D140">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C141" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D141">
-        <v>0.2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C142" t="s">
+        <v>22</v>
       </c>
       <c r="D142">
-        <v>0.55000000000000004</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
-        <v>10</v>
-      </c>
-      <c r="C143" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D143">
-        <v>4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
+        <v>10</v>
+      </c>
+      <c r="C144" t="s">
+        <v>11</v>
+      </c>
+      <c r="D144">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="145" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B145" t="s">
         <v>44</v>
       </c>
-      <c r="C144" t="s">
+      <c r="C145" t="s">
         <v>45</v>
       </c>
-      <c r="D144">
+      <c r="D145">
         <v>0.2</v>
       </c>
     </row>
@@ -4403,7 +4448,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E1">
         <v>2020</v>
@@ -4423,10 +4468,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
         <v>91</v>
-      </c>
-      <c r="C2" t="s">
-        <v>92</v>
       </c>
       <c r="D2">
         <v>0.7</v>
@@ -4438,10 +4483,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>0.7</v>
@@ -4453,13 +4498,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
         <v>91</v>
-      </c>
-      <c r="C4" t="s">
-        <v>92</v>
       </c>
       <c r="D4">
         <v>0.7</v>
@@ -4471,10 +4516,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>0.7</v>
@@ -4489,10 +4534,10 @@
         <v>59</v>
       </c>
       <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
         <v>91</v>
-      </c>
-      <c r="C6" t="s">
-        <v>92</v>
       </c>
       <c r="D6">
         <v>0.7</v>
@@ -4504,10 +4549,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>0.7</v>
@@ -4522,10 +4567,10 @@
         <v>61</v>
       </c>
       <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
         <v>91</v>
-      </c>
-      <c r="C8" t="s">
-        <v>92</v>
       </c>
       <c r="D8">
         <v>0.7</v>
@@ -4537,10 +4582,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>0.7</v>
@@ -4555,10 +4600,10 @@
         <v>43</v>
       </c>
       <c r="B10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" t="s">
         <v>91</v>
-      </c>
-      <c r="C10" t="s">
-        <v>92</v>
       </c>
       <c r="D10">
         <v>0.7</v>
@@ -4570,10 +4615,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>0.7</v>
@@ -4588,10 +4633,10 @@
         <v>53</v>
       </c>
       <c r="B12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" t="s">
         <v>91</v>
-      </c>
-      <c r="C12" t="s">
-        <v>92</v>
       </c>
       <c r="D12">
         <v>0.7</v>
@@ -4603,10 +4648,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>0.7</v>
@@ -4621,10 +4666,10 @@
         <v>54</v>
       </c>
       <c r="B14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" t="s">
         <v>91</v>
-      </c>
-      <c r="C14" t="s">
-        <v>92</v>
       </c>
       <c r="D14">
         <v>0.7</v>
@@ -4636,10 +4681,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>0.7</v>
@@ -4651,13 +4696,13 @@
     </row>
     <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" t="s">
         <v>95</v>
-      </c>
-      <c r="B16" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" t="s">
-        <v>96</v>
       </c>
       <c r="D16" s="2">
         <f>40*0.1</f>
@@ -4670,10 +4715,10 @@
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D17" s="2">
         <f t="shared" ref="D17:D21" si="0">40*0.1</f>
@@ -4689,10 +4734,10 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D18" s="2">
         <f t="shared" si="0"/>
@@ -4705,10 +4750,10 @@
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D19" s="2">
         <f t="shared" si="0"/>
@@ -4721,13 +4766,13 @@
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D20" s="2">
         <f t="shared" si="0"/>
@@ -4740,10 +4785,10 @@
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D21" s="2">
         <f t="shared" si="0"/>
@@ -4756,13 +4801,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" t="s">
         <v>91</v>
-      </c>
-      <c r="C22" t="s">
-        <v>92</v>
       </c>
       <c r="D22">
         <v>0.7</v>
@@ -4770,10 +4815,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D23">
         <v>0.7</v>
@@ -4781,13 +4826,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" t="s">
         <v>91</v>
-      </c>
-      <c r="C24" t="s">
-        <v>92</v>
       </c>
       <c r="D24">
         <v>0.7</v>
@@ -4795,10 +4840,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D25">
         <v>0.7</v>
@@ -4806,13 +4851,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" t="s">
         <v>91</v>
-      </c>
-      <c r="C26" t="s">
-        <v>92</v>
       </c>
       <c r="D26">
         <v>0.7</v>
@@ -4820,10 +4865,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D27">
         <v>0.7</v>

</xml_diff>

<commit_message>
Changes to excel and README
</commit_message>
<xml_diff>
--- a/Group Assignment MfT/input_databases/default/technologies.xlsx
+++ b/Group Assignment MfT/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling_for_transitions_Group/Group Assignment MfT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEAD918F-2CF4-A748-8E08-59B83AD8A7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{541339A1-A0D4-9B45-8235-F25DAB26D78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="107">
   <si>
     <t>Technology</t>
   </si>
@@ -260,9 +260,6 @@
     <t>Biomass + CCS (BECCS), net negative emissions</t>
   </si>
   <si>
-    <t>Residential gas boiler</t>
-  </si>
-  <si>
     <t>Gas boiler to generate space and water heating</t>
   </si>
   <si>
@@ -341,9 +338,6 @@
     <t>Industrial HTP - fossil - existing</t>
   </si>
   <si>
-    <t>Residential gas boiler - existing</t>
-  </si>
-  <si>
     <t>Generic industrial machinery running on fossil energy - existing base</t>
   </si>
   <si>
@@ -357,6 +351,18 @@
   </si>
   <si>
     <t>Subsidy</t>
+  </si>
+  <si>
+    <t>Residential gas boiler high</t>
+  </si>
+  <si>
+    <t>Residential gas boiler low</t>
+  </si>
+  <si>
+    <t>Residential gas boiler high - existing</t>
+  </si>
+  <si>
+    <t>Residential gas boiler low - existing</t>
   </si>
 </sst>
 </file>
@@ -691,7 +697,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2AEF3F7-9EA9-4235-9872-78FDC34EDD32}">
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -1455,13 +1461,13 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="B71" t="s">
         <v>49</v>
       </c>
       <c r="E71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
@@ -1502,7 +1508,7 @@
         <v>9</v>
       </c>
       <c r="E75" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -1520,80 +1526,80 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>104</v>
+      </c>
       <c r="B77" t="s">
-        <v>66</v>
-      </c>
-      <c r="C77" t="s">
-        <v>32</v>
-      </c>
-      <c r="D77" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="E77" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>74</v>
-      </c>
       <c r="B78" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E78" t="s">
-        <v>75</v>
+        <v>39</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E79" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C80" t="s">
+        <v>29</v>
       </c>
       <c r="E80" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C81" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D81" t="s">
+        <v>9</v>
       </c>
       <c r="E81" t="s">
-        <v>34</v>
+        <v>100</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C82" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D82" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E82" t="s">
-        <v>103</v>
+        <v>48</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B83" t="s">
         <v>49</v>
       </c>
       <c r="E83" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -1601,7 +1607,7 @@
         <v>16</v>
       </c>
       <c r="E84" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -1620,7 +1626,7 @@
         <v>29</v>
       </c>
       <c r="E86" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -1634,125 +1640,122 @@
         <v>9</v>
       </c>
       <c r="E87" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>75</v>
+      </c>
       <c r="B88" t="s">
-        <v>46</v>
-      </c>
-      <c r="C88" t="s">
-        <v>47</v>
-      </c>
-      <c r="D88" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E88" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>80</v>
-      </c>
       <c r="B89" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E89" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E90" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B91" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C91" t="s">
+        <v>29</v>
       </c>
       <c r="E91" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B92" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C92" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D92" t="s">
+        <v>9</v>
       </c>
       <c r="E92" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C93" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D93" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E93" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B94" t="s">
-        <v>46</v>
-      </c>
-      <c r="C94" t="s">
-        <v>47</v>
-      </c>
-      <c r="D94" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E94" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B95" t="s">
-        <v>66</v>
-      </c>
-      <c r="C95" t="s">
-        <v>67</v>
-      </c>
-      <c r="D95" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="E95" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B96" t="s">
-        <v>52</v>
-      </c>
-      <c r="E96">
-        <v>2030</v>
+        <v>24</v>
+      </c>
+      <c r="E96" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>82</v>
-      </c>
       <c r="B97" t="s">
-        <v>49</v>
+        <v>28</v>
+      </c>
+      <c r="C97" t="s">
+        <v>29</v>
       </c>
       <c r="E97" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B98" t="s">
-        <v>16</v>
+        <v>31</v>
+      </c>
+      <c r="C98" t="s">
+        <v>32</v>
+      </c>
+      <c r="D98" t="s">
+        <v>9</v>
       </c>
       <c r="E98" t="s">
         <v>78</v>
@@ -1760,46 +1763,49 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B99" t="s">
-        <v>24</v>
+        <v>46</v>
+      </c>
+      <c r="C99" t="s">
+        <v>47</v>
+      </c>
+      <c r="D99" t="s">
+        <v>44</v>
       </c>
       <c r="E99" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="C100" t="s">
-        <v>29</v>
+        <v>67</v>
+      </c>
+      <c r="D100" t="s">
+        <v>68</v>
       </c>
       <c r="E100" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
-        <v>31</v>
-      </c>
-      <c r="C101" t="s">
-        <v>32</v>
-      </c>
-      <c r="D101" t="s">
-        <v>9</v>
-      </c>
-      <c r="E101" t="s">
-        <v>79</v>
+        <v>52</v>
+      </c>
+      <c r="E101">
+        <v>2030</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B102" t="s">
         <v>49</v>
       </c>
       <c r="E102" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
@@ -1807,7 +1813,7 @@
         <v>16</v>
       </c>
       <c r="E103" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
@@ -1826,7 +1832,7 @@
         <v>29</v>
       </c>
       <c r="E105" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -1840,172 +1846,172 @@
         <v>9</v>
       </c>
       <c r="E106" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>83</v>
+      </c>
       <c r="B107" t="s">
-        <v>46</v>
-      </c>
-      <c r="C107" t="s">
-        <v>47</v>
-      </c>
-      <c r="D107" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E107" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
-        <v>87</v>
-      </c>
       <c r="B108" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E108" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E109" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C110" t="s">
+        <v>29</v>
       </c>
       <c r="E110" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C111" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D111" t="s">
+        <v>9</v>
       </c>
       <c r="E111" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C112" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D112" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E112" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
-        <v>46</v>
-      </c>
-      <c r="C113" t="s">
-        <v>47</v>
-      </c>
-      <c r="D113" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E113" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
-        <v>66</v>
-      </c>
-      <c r="C114" t="s">
-        <v>67</v>
-      </c>
-      <c r="D114" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="E114" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
-        <v>52</v>
-      </c>
-      <c r="E115">
-        <v>2030</v>
+        <v>24</v>
+      </c>
+      <c r="E115" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
-        <v>94</v>
-      </c>
       <c r="B116" t="s">
-        <v>49</v>
+        <v>28</v>
+      </c>
+      <c r="C116" t="s">
+        <v>29</v>
       </c>
       <c r="E116" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
-        <v>16</v>
+        <v>31</v>
+      </c>
+      <c r="C117" t="s">
+        <v>32</v>
+      </c>
+      <c r="D117" t="s">
+        <v>9</v>
       </c>
       <c r="E117" t="s">
-        <v>19</v>
+        <v>85</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>24</v>
+        <v>46</v>
+      </c>
+      <c r="C118" t="s">
+        <v>47</v>
+      </c>
+      <c r="D118" t="s">
+        <v>44</v>
       </c>
       <c r="E118" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="C119" t="s">
-        <v>29</v>
+        <v>67</v>
+      </c>
+      <c r="D119" t="s">
+        <v>68</v>
       </c>
       <c r="E119" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
-        <v>31</v>
-      </c>
-      <c r="C120" t="s">
-        <v>32</v>
-      </c>
-      <c r="D120" t="s">
-        <v>9</v>
-      </c>
-      <c r="E120" t="s">
-        <v>35</v>
+        <v>52</v>
+      </c>
+      <c r="E120">
+        <v>2030</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B121" t="s">
         <v>49</v>
       </c>
       <c r="E121" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
@@ -2032,7 +2038,7 @@
         <v>29</v>
       </c>
       <c r="E124" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
@@ -2050,294 +2056,398 @@
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>95</v>
+      </c>
       <c r="B126" t="s">
-        <v>46</v>
-      </c>
-      <c r="C126" t="s">
-        <v>47</v>
-      </c>
-      <c r="D126" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E126" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>93</v>
-      </c>
       <c r="B127" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E127" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E128" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C129" t="s">
+        <v>29</v>
       </c>
       <c r="E129" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C130" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D130" t="s">
+        <v>9</v>
       </c>
       <c r="E130" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C131" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D131" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E131" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
+        <v>92</v>
+      </c>
       <c r="B132" t="s">
-        <v>46</v>
-      </c>
-      <c r="C132" t="s">
-        <v>47</v>
-      </c>
-      <c r="D132" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E132" t="s">
-        <v>48</v>
+        <v>5</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
-        <v>99</v>
-      </c>
       <c r="B133" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E133" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E134" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C135" t="s">
+        <v>29</v>
       </c>
       <c r="E135" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C136" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D136" t="s">
+        <v>9</v>
       </c>
       <c r="E136" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C137" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D137" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E137" t="s">
-        <v>102</v>
+        <v>48</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
+        <v>105</v>
+      </c>
       <c r="B138" t="s">
-        <v>46</v>
-      </c>
-      <c r="C138" t="s">
-        <v>47</v>
-      </c>
-      <c r="D138" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E138" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
-        <v>66</v>
-      </c>
-      <c r="C139" t="s">
-        <v>32</v>
-      </c>
-      <c r="D139" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E139" t="s">
-        <v>103</v>
+        <v>39</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
-        <v>97</v>
-      </c>
       <c r="B140" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E140" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
-        <v>16</v>
+        <v>28</v>
+      </c>
+      <c r="C141" t="s">
+        <v>29</v>
       </c>
       <c r="E141" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="C142" t="s">
+        <v>32</v>
+      </c>
+      <c r="D142" t="s">
+        <v>9</v>
       </c>
       <c r="E142" t="s">
-        <v>25</v>
+        <v>101</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C143" t="s">
-        <v>29</v>
+        <v>47</v>
+      </c>
+      <c r="D143" t="s">
+        <v>44</v>
       </c>
       <c r="E143" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
+        <v>106</v>
+      </c>
       <c r="B144" t="s">
-        <v>31</v>
-      </c>
-      <c r="C144" t="s">
-        <v>32</v>
-      </c>
-      <c r="D144" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="E144" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
-        <v>46</v>
-      </c>
-      <c r="C145" t="s">
-        <v>47</v>
-      </c>
-      <c r="D145" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="E145" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
-        <v>98</v>
-      </c>
       <c r="B146" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E146" t="s">
-        <v>101</v>
+        <v>25</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
-        <v>16</v>
+        <v>28</v>
+      </c>
+      <c r="C147" t="s">
+        <v>29</v>
       </c>
       <c r="E147" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="C148" t="s">
+        <v>32</v>
+      </c>
+      <c r="D148" t="s">
+        <v>9</v>
       </c>
       <c r="E148" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B149" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C149" t="s">
-        <v>29</v>
+        <v>47</v>
+      </c>
+      <c r="D149" t="s">
+        <v>44</v>
       </c>
       <c r="E149" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A150" t="s">
+        <v>96</v>
+      </c>
       <c r="B150" t="s">
-        <v>31</v>
-      </c>
-      <c r="C150" t="s">
-        <v>32</v>
-      </c>
-      <c r="D150" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="E150" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B151" t="s">
+        <v>16</v>
+      </c>
+      <c r="E151" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B152" t="s">
+        <v>24</v>
+      </c>
+      <c r="E152" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B153" t="s">
+        <v>28</v>
+      </c>
+      <c r="C153" t="s">
+        <v>29</v>
+      </c>
+      <c r="E153" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B154" t="s">
+        <v>31</v>
+      </c>
+      <c r="C154" t="s">
+        <v>32</v>
+      </c>
+      <c r="D154" t="s">
+        <v>9</v>
+      </c>
+      <c r="E154" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B155" t="s">
         <v>46</v>
       </c>
-      <c r="C151" t="s">
+      <c r="C155" t="s">
         <v>47</v>
       </c>
-      <c r="D151" t="s">
+      <c r="D155" t="s">
         <v>44</v>
       </c>
-      <c r="E151" t="s">
+      <c r="E155" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A156" t="s">
+        <v>97</v>
+      </c>
+      <c r="B156" t="s">
+        <v>49</v>
+      </c>
+      <c r="E156" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B157" t="s">
+        <v>16</v>
+      </c>
+      <c r="E157" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B158" t="s">
+        <v>24</v>
+      </c>
+      <c r="E158" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B159" t="s">
+        <v>28</v>
+      </c>
+      <c r="C159" t="s">
+        <v>29</v>
+      </c>
+      <c r="E159" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B160" t="s">
+        <v>31</v>
+      </c>
+      <c r="C160" t="s">
+        <v>32</v>
+      </c>
+      <c r="D160" t="s">
+        <v>9</v>
+      </c>
+      <c r="E160" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="161" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B161" t="s">
+        <v>46</v>
+      </c>
+      <c r="C161" t="s">
+        <v>47</v>
+      </c>
+      <c r="D161" t="s">
+        <v>44</v>
+      </c>
+      <c r="E161" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2350,7 +2460,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -3416,7 +3526,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
@@ -3489,7 +3599,7 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="B74" t="s">
         <v>6</v>
@@ -3498,85 +3608,71 @@
         <v>21</v>
       </c>
       <c r="D74">
-        <v>2200</v>
-      </c>
-      <c r="E74">
-        <v>2000</v>
+        <v>200</v>
+      </c>
+      <c r="G74">
+        <v>150</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
-        <v>104</v>
+        <v>7</v>
       </c>
       <c r="C75" t="s">
         <v>21</v>
       </c>
       <c r="D75">
-        <v>200</v>
-      </c>
-      <c r="E75">
-        <v>200</v>
+        <f>D74*0.05</f>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C76" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D76">
-        <f>D74*0.05</f>
-        <v>110</v>
-      </c>
-      <c r="E76">
-        <f>E75*0.05</f>
-        <v>10</v>
-      </c>
-      <c r="G76">
-        <f>G75*0.05</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
-        <v>8</v>
-      </c>
-      <c r="C77" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="D77">
-        <v>0</v>
+        <v>0.9</v>
+      </c>
+      <c r="E77">
+        <v>0.95</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="C78" t="s">
+        <v>11</v>
       </c>
       <c r="D78">
-        <v>3</v>
-      </c>
-      <c r="E78">
-        <v>4</v>
-      </c>
-      <c r="G78">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="C79" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="D79">
-        <v>12</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B80" t="s">
         <v>6</v>
@@ -3585,84 +3681,85 @@
         <v>21</v>
       </c>
       <c r="D80">
-        <v>450</v>
-      </c>
-      <c r="G80">
-        <v>300</v>
+        <v>2200</v>
+      </c>
+      <c r="E80">
+        <v>2000</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
-        <v>7</v>
+        <v>102</v>
       </c>
       <c r="C81" t="s">
         <v>21</v>
       </c>
       <c r="D81">
-        <f>D80*0.05</f>
-        <v>22.5</v>
-      </c>
-      <c r="G81">
-        <f>G80*0.05</f>
-        <v>15</v>
+        <v>200</v>
+      </c>
+      <c r="E81">
+        <v>200</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B82" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C82" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D82">
-        <v>0.2</v>
+        <f>D80*0.05</f>
+        <v>110</v>
+      </c>
+      <c r="E82">
+        <f>E81*0.05</f>
+        <v>10</v>
       </c>
       <c r="G82">
-        <v>0.2</v>
+        <f>G81*0.05</f>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B83" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>22</v>
       </c>
       <c r="D83">
-        <v>0.85</v>
-      </c>
-      <c r="G83">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B84" t="s">
-        <v>10</v>
-      </c>
-      <c r="C84" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D84">
-        <v>20</v>
+        <v>3</v>
+      </c>
+      <c r="E84">
+        <v>4</v>
       </c>
       <c r="G84">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B85" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="C85" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="D85">
-        <v>0.2</v>
-      </c>
-      <c r="G85">
-        <v>0.2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B86" t="s">
         <v>6</v>
@@ -3671,11 +3768,10 @@
         <v>21</v>
       </c>
       <c r="D86">
-        <f>D80*2</f>
-        <v>900</v>
+        <v>450</v>
       </c>
       <c r="G86">
-        <v>500</v>
+        <v>300</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
@@ -3687,11 +3783,11 @@
       </c>
       <c r="D87">
         <f>D86*0.05</f>
-        <v>45</v>
+        <v>22.5</v>
       </c>
       <c r="G87">
         <f>G86*0.05</f>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -3702,10 +3798,10 @@
         <v>22</v>
       </c>
       <c r="D88">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G88">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
@@ -3713,10 +3809,10 @@
         <v>9</v>
       </c>
       <c r="D89">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="G89">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -3741,191 +3837,192 @@
         <v>45</v>
       </c>
       <c r="D91">
+        <v>0.2</v>
+      </c>
+      <c r="G91">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>79</v>
+      </c>
+      <c r="B92" t="s">
+        <v>6</v>
+      </c>
+      <c r="C92" t="s">
+        <v>21</v>
+      </c>
+      <c r="D92">
+        <f>D86*2</f>
+        <v>900</v>
+      </c>
+      <c r="G92">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B93" t="s">
+        <v>7</v>
+      </c>
+      <c r="C93" t="s">
+        <v>21</v>
+      </c>
+      <c r="D93">
+        <f>D92*0.05</f>
+        <v>45</v>
+      </c>
+      <c r="G93">
+        <f>G92*0.05</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94" t="s">
+        <v>22</v>
+      </c>
+      <c r="D94">
+        <v>0.4</v>
+      </c>
+      <c r="G94">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B95" t="s">
+        <v>9</v>
+      </c>
+      <c r="D95">
+        <v>0.8</v>
+      </c>
+      <c r="G95">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B96" t="s">
+        <v>10</v>
+      </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96">
+        <v>20</v>
+      </c>
+      <c r="G96">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B97" t="s">
+        <v>44</v>
+      </c>
+      <c r="C97" t="s">
+        <v>45</v>
+      </c>
+      <c r="D97">
         <f>0.2*0.15</f>
         <v>0.03</v>
       </c>
-      <c r="G91">
+      <c r="G97">
         <f>0.2*0.1</f>
         <v>2.0000000000000004E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B92" t="s">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B98" t="s">
         <v>68</v>
       </c>
-      <c r="C92" t="s">
+      <c r="C98" t="s">
         <v>45</v>
       </c>
-      <c r="D92">
+      <c r="D98">
         <f>0.2*0.85</f>
         <v>0.17</v>
       </c>
-      <c r="G92">
+      <c r="G98">
         <f>0.2*0.9</f>
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>82</v>
-      </c>
-      <c r="B93" t="s">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>81</v>
+      </c>
+      <c r="B99" t="s">
         <v>6</v>
-      </c>
-      <c r="C93" t="s">
-        <v>21</v>
-      </c>
-      <c r="D93">
-        <v>350</v>
-      </c>
-      <c r="G93">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B94" t="s">
-        <v>7</v>
-      </c>
-      <c r="C94" t="s">
-        <v>21</v>
-      </c>
-      <c r="D94">
-        <f>D93*0.05</f>
-        <v>17.5</v>
-      </c>
-      <c r="G94">
-        <f>G93*0.05</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B95" t="s">
-        <v>8</v>
-      </c>
-      <c r="C95" t="s">
-        <v>22</v>
-      </c>
-      <c r="D95">
-        <v>0.2</v>
-      </c>
-      <c r="G95">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B96" t="s">
-        <v>9</v>
-      </c>
-      <c r="D96">
-        <v>0.95</v>
-      </c>
-      <c r="G96">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B97" t="s">
-        <v>10</v>
-      </c>
-      <c r="C97" t="s">
-        <v>11</v>
-      </c>
-      <c r="D97">
-        <v>15</v>
-      </c>
-      <c r="G97">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>84</v>
-      </c>
-      <c r="B98" t="s">
-        <v>6</v>
-      </c>
-      <c r="C98" t="s">
-        <v>21</v>
-      </c>
-      <c r="D98">
-        <v>900</v>
-      </c>
-      <c r="G98">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B99" t="s">
-        <v>7</v>
       </c>
       <c r="C99" t="s">
         <v>21</v>
       </c>
       <c r="D99">
-        <f>D98*0.05</f>
-        <v>45</v>
+        <v>350</v>
       </c>
       <c r="G99">
-        <f>G98*0.05</f>
-        <v>20</v>
+        <v>100</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B100" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C100" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D100">
-        <v>0.2</v>
+        <f>D99*0.05</f>
+        <v>17.5</v>
       </c>
       <c r="G100">
-        <v>0.2</v>
+        <f>G99*0.05</f>
+        <v>5</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B101" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C101" t="s">
+        <v>22</v>
       </c>
       <c r="D101">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="G101">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B102" t="s">
-        <v>10</v>
-      </c>
-      <c r="C102" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D102">
-        <v>20</v>
+        <v>0.95</v>
       </c>
       <c r="G102">
-        <v>20</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="C103" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="D103">
-        <v>0.2</v>
+        <v>15</v>
       </c>
       <c r="G103">
-        <v>0.2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B104" t="s">
         <v>6</v>
@@ -3934,11 +4031,10 @@
         <v>21</v>
       </c>
       <c r="D104">
-        <f>D98*2</f>
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="G104">
-        <v>1000</v>
+        <v>400</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -3950,11 +4046,11 @@
       </c>
       <c r="D105">
         <f>D104*0.05</f>
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="G105">
         <f>G104*0.05</f>
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
@@ -3965,10 +4061,10 @@
         <v>22</v>
       </c>
       <c r="D106">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G106">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
@@ -3976,10 +4072,10 @@
         <v>9</v>
       </c>
       <c r="D107">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G107">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
@@ -4004,105 +4100,123 @@
         <v>45</v>
       </c>
       <c r="D109">
+        <v>0.2</v>
+      </c>
+      <c r="G109">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>86</v>
+      </c>
+      <c r="B110" t="s">
+        <v>6</v>
+      </c>
+      <c r="C110" t="s">
+        <v>21</v>
+      </c>
+      <c r="D110">
+        <f>D104*2</f>
+        <v>1800</v>
+      </c>
+      <c r="G110">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B111" t="s">
+        <v>7</v>
+      </c>
+      <c r="C111" t="s">
+        <v>21</v>
+      </c>
+      <c r="D111">
+        <f>D110*0.05</f>
+        <v>90</v>
+      </c>
+      <c r="G111">
+        <f>G110*0.05</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B112" t="s">
+        <v>8</v>
+      </c>
+      <c r="C112" t="s">
+        <v>22</v>
+      </c>
+      <c r="D112">
+        <v>0.4</v>
+      </c>
+      <c r="G112">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B113" t="s">
+        <v>9</v>
+      </c>
+      <c r="D113">
+        <v>0.5</v>
+      </c>
+      <c r="G113">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B114" t="s">
+        <v>10</v>
+      </c>
+      <c r="C114" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114">
+        <v>20</v>
+      </c>
+      <c r="G114">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B115" t="s">
+        <v>44</v>
+      </c>
+      <c r="C115" t="s">
+        <v>45</v>
+      </c>
+      <c r="D115">
         <f>0.2*0.15</f>
         <v>0.03</v>
       </c>
-      <c r="G109">
+      <c r="G115">
         <f>0.2*0.1</f>
         <v>2.0000000000000004E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B110" t="s">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B116" t="s">
         <v>68</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C116" t="s">
         <v>45</v>
       </c>
-      <c r="D110">
+      <c r="D116">
         <f>0.2*0.85</f>
         <v>0.17</v>
       </c>
-      <c r="G110">
+      <c r="G116">
         <f>0.2*0.9</f>
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>94</v>
-      </c>
-      <c r="B111" t="s">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>93</v>
+      </c>
+      <c r="B117" t="s">
         <v>6</v>
-      </c>
-      <c r="C111" t="s">
-        <v>23</v>
-      </c>
-      <c r="D111">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B112" t="s">
-        <v>7</v>
-      </c>
-      <c r="C112" t="s">
-        <v>23</v>
-      </c>
-      <c r="D112">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B113" t="s">
-        <v>8</v>
-      </c>
-      <c r="C113" t="s">
-        <v>22</v>
-      </c>
-      <c r="D113">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B114" t="s">
-        <v>9</v>
-      </c>
-      <c r="C114" t="s">
-        <v>20</v>
-      </c>
-      <c r="D114">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B115" t="s">
-        <v>10</v>
-      </c>
-      <c r="C115" t="s">
-        <v>11</v>
-      </c>
-      <c r="D115">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
-        <v>96</v>
-      </c>
-      <c r="B116" t="s">
-        <v>6</v>
-      </c>
-      <c r="C116" t="s">
-        <v>23</v>
-      </c>
-      <c r="D116">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B117" t="s">
-        <v>7</v>
       </c>
       <c r="C117" t="s">
         <v>23</v>
@@ -4111,76 +4225,76 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C118" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D118">
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C119" t="s">
+        <v>22</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B120" t="s">
+        <v>9</v>
+      </c>
+      <c r="C120" t="s">
         <v>20</v>
       </c>
-      <c r="D119">
+      <c r="D120">
         <v>2.5</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B120" t="s">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B121" t="s">
         <v>10</v>
       </c>
-      <c r="C120" t="s">
+      <c r="C121" t="s">
         <v>11</v>
       </c>
-      <c r="D120">
+      <c r="D121">
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B121" t="s">
-        <v>44</v>
-      </c>
-      <c r="C121" t="s">
-        <v>45</v>
-      </c>
-      <c r="D121">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B122" t="s">
         <v>6</v>
       </c>
       <c r="C122" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D122">
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
         <v>7</v>
       </c>
       <c r="C123" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D123">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
         <v>8</v>
       </c>
@@ -4188,18 +4302,21 @@
         <v>22</v>
       </c>
       <c r="D124">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
         <v>9</v>
       </c>
+      <c r="C125" t="s">
+        <v>20</v>
+      </c>
       <c r="D125">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
         <v>10</v>
       </c>
@@ -4210,7 +4327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
         <v>44</v>
       </c>
@@ -4218,12 +4335,12 @@
         <v>45</v>
       </c>
       <c r="D127">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B128" t="s">
         <v>6</v>
@@ -4243,8 +4360,7 @@
         <v>21</v>
       </c>
       <c r="D129">
-        <f>D128*0.05</f>
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
@@ -4255,7 +4371,7 @@
         <v>22</v>
       </c>
       <c r="D130">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
@@ -4263,7 +4379,7 @@
         <v>9</v>
       </c>
       <c r="D131">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
@@ -4290,7 +4406,7 @@
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B134" t="s">
         <v>6</v>
@@ -4310,7 +4426,8 @@
         <v>21</v>
       </c>
       <c r="D135">
-        <v>20</v>
+        <f>D134*0.05</f>
+        <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.2">
@@ -4321,7 +4438,7 @@
         <v>22</v>
       </c>
       <c r="D136">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.2">
@@ -4329,7 +4446,7 @@
         <v>9</v>
       </c>
       <c r="D137">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
@@ -4356,7 +4473,7 @@
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B140" t="s">
         <v>6</v>
@@ -4376,7 +4493,8 @@
         <v>21</v>
       </c>
       <c r="D141">
-        <v>40</v>
+        <f>D140*0.05</f>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
@@ -4387,7 +4505,7 @@
         <v>22</v>
       </c>
       <c r="D142">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
@@ -4395,7 +4513,7 @@
         <v>9</v>
       </c>
       <c r="D143">
-        <v>0.55000000000000004</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
@@ -4409,7 +4527,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="145" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
         <v>44</v>
       </c>
@@ -4417,6 +4535,138 @@
         <v>45</v>
       </c>
       <c r="D145">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
+        <v>96</v>
+      </c>
+      <c r="B146" t="s">
+        <v>6</v>
+      </c>
+      <c r="C146" t="s">
+        <v>21</v>
+      </c>
+      <c r="D146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B147" t="s">
+        <v>7</v>
+      </c>
+      <c r="C147" t="s">
+        <v>21</v>
+      </c>
+      <c r="D147">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B148" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" t="s">
+        <v>22</v>
+      </c>
+      <c r="D148">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B149" t="s">
+        <v>9</v>
+      </c>
+      <c r="D149">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B150" t="s">
+        <v>10</v>
+      </c>
+      <c r="C150" t="s">
+        <v>11</v>
+      </c>
+      <c r="D150">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B151" t="s">
+        <v>44</v>
+      </c>
+      <c r="C151" t="s">
+        <v>45</v>
+      </c>
+      <c r="D151">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
+        <v>97</v>
+      </c>
+      <c r="B152" t="s">
+        <v>6</v>
+      </c>
+      <c r="C152" t="s">
+        <v>21</v>
+      </c>
+      <c r="D152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B153" t="s">
+        <v>7</v>
+      </c>
+      <c r="C153" t="s">
+        <v>21</v>
+      </c>
+      <c r="D153">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B154" t="s">
+        <v>8</v>
+      </c>
+      <c r="C154" t="s">
+        <v>22</v>
+      </c>
+      <c r="D154">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B155" t="s">
+        <v>9</v>
+      </c>
+      <c r="D155">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B156" t="s">
+        <v>10</v>
+      </c>
+      <c r="C156" t="s">
+        <v>11</v>
+      </c>
+      <c r="D156">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B157" t="s">
+        <v>44</v>
+      </c>
+      <c r="C157" t="s">
+        <v>45</v>
+      </c>
+      <c r="D157">
         <v>0.2</v>
       </c>
     </row>
@@ -4448,7 +4698,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E1">
         <v>2020</v>
@@ -4468,10 +4718,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
         <v>90</v>
-      </c>
-      <c r="C2" t="s">
-        <v>91</v>
       </c>
       <c r="D2">
         <v>0.7</v>
@@ -4483,10 +4733,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D3">
         <v>0.7</v>
@@ -4498,13 +4748,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
         <v>90</v>
-      </c>
-      <c r="C4" t="s">
-        <v>91</v>
       </c>
       <c r="D4">
         <v>0.7</v>
@@ -4516,10 +4766,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D5">
         <v>0.7</v>
@@ -4534,10 +4784,10 @@
         <v>59</v>
       </c>
       <c r="B6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" t="s">
         <v>90</v>
-      </c>
-      <c r="C6" t="s">
-        <v>91</v>
       </c>
       <c r="D6">
         <v>0.7</v>
@@ -4549,10 +4799,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D7">
         <v>0.7</v>
@@ -4567,10 +4817,10 @@
         <v>61</v>
       </c>
       <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
         <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>91</v>
       </c>
       <c r="D8">
         <v>0.7</v>
@@ -4582,10 +4832,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9">
         <v>0.7</v>
@@ -4600,10 +4850,10 @@
         <v>43</v>
       </c>
       <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
         <v>90</v>
-      </c>
-      <c r="C10" t="s">
-        <v>91</v>
       </c>
       <c r="D10">
         <v>0.7</v>
@@ -4615,10 +4865,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D11">
         <v>0.7</v>
@@ -4633,10 +4883,10 @@
         <v>53</v>
       </c>
       <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" t="s">
         <v>90</v>
-      </c>
-      <c r="C12" t="s">
-        <v>91</v>
       </c>
       <c r="D12">
         <v>0.7</v>
@@ -4648,10 +4898,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D13">
         <v>0.7</v>
@@ -4666,10 +4916,10 @@
         <v>54</v>
       </c>
       <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" t="s">
         <v>90</v>
-      </c>
-      <c r="C14" t="s">
-        <v>91</v>
       </c>
       <c r="D14">
         <v>0.7</v>
@@ -4681,10 +4931,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D15">
         <v>0.7</v>
@@ -4696,13 +4946,13 @@
     </row>
     <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
         <v>94</v>
-      </c>
-      <c r="B16" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" t="s">
-        <v>95</v>
       </c>
       <c r="D16" s="2">
         <f>40*0.1</f>
@@ -4715,10 +4965,10 @@
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D17" s="2">
         <f t="shared" ref="D17:D21" si="0">40*0.1</f>
@@ -4734,10 +4984,10 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D18" s="2">
         <f t="shared" si="0"/>
@@ -4750,10 +5000,10 @@
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D19" s="2">
         <f t="shared" si="0"/>
@@ -4766,13 +5016,13 @@
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D20" s="2">
         <f t="shared" si="0"/>
@@ -4785,10 +5035,10 @@
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D21" s="2">
         <f t="shared" si="0"/>
@@ -4801,13 +5051,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B22" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" t="s">
         <v>90</v>
-      </c>
-      <c r="C22" t="s">
-        <v>91</v>
       </c>
       <c r="D22">
         <v>0.7</v>
@@ -4815,10 +5065,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D23">
         <v>0.7</v>
@@ -4826,13 +5076,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" t="s">
         <v>90</v>
-      </c>
-      <c r="C24" t="s">
-        <v>91</v>
       </c>
       <c r="D24">
         <v>0.7</v>
@@ -4840,10 +5090,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D25">
         <v>0.7</v>
@@ -4851,13 +5101,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" t="s">
         <v>90</v>
-      </c>
-      <c r="C26" t="s">
-        <v>91</v>
       </c>
       <c r="D26">
         <v>0.7</v>
@@ -4865,10 +5115,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D27">
         <v>0.7</v>

</xml_diff>

<commit_message>
Fixed error subsidy and added graphs, still to be finished
</commit_message>
<xml_diff>
--- a/Group Assignment MfT/input_databases/default/technologies.xlsx
+++ b/Group Assignment MfT/input_databases/default/technologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling_for_transitions_Group/Group Assignment MfT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{541339A1-A0D4-9B45-8235-F25DAB26D78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{47809E97-A945-7449-99AC-D48D7B4388E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -3681,10 +3681,10 @@
         <v>21</v>
       </c>
       <c r="D80">
-        <v>2200</v>
+        <v>4000</v>
       </c>
       <c r="E80">
-        <v>2000</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -3695,10 +3695,16 @@
         <v>21</v>
       </c>
       <c r="D81">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="E81">
-        <v>200</v>
+        <v>2000</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="G81">
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -3710,11 +3716,11 @@
       </c>
       <c r="D82">
         <f>D80*0.05</f>
-        <v>110</v>
+        <v>200</v>
       </c>
       <c r="E82">
         <f>E81*0.05</f>
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G82">
         <f>G81*0.05</f>

</xml_diff>

<commit_message>
Added heat maps + changes to subsidy_growth
</commit_message>
<xml_diff>
--- a/Group Assignment MfT/input_databases/default/technologies.xlsx
+++ b/Group Assignment MfT/input_databases/default/technologies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling_for_transitions_Group/Group Assignment MfT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47809E97-A945-7449-99AC-D48D7B4388E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{211B4C32-4B70-D246-8F70-E8ED390293AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3535,10 +3535,10 @@
         <v>21</v>
       </c>
       <c r="D68">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="G68">
-        <v>150</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="D69">
         <f>D68*0.05</f>
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -3608,10 +3608,10 @@
         <v>21</v>
       </c>
       <c r="D74">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="G74">
-        <v>150</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D75">
         <f>D74*0.05</f>
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -3686,6 +3686,12 @@
       <c r="E80">
         <v>3800</v>
       </c>
+      <c r="F80">
+        <v>3610</v>
+      </c>
+      <c r="G80">
+        <v>3429</v>
+      </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B81" t="s">
@@ -3695,16 +3701,20 @@
         <v>21</v>
       </c>
       <c r="D81">
-        <v>2000</v>
+        <f>D80*0.3</f>
+        <v>1200</v>
       </c>
       <c r="E81">
-        <v>2000</v>
+        <f>E80*0.3</f>
+        <v>1140</v>
       </c>
       <c r="F81">
-        <v>0</v>
+        <f t="shared" ref="F81:G81" si="3">F80*0.3</f>
+        <v>1083</v>
       </c>
       <c r="G81">
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>1028.7</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -3715,16 +3725,8 @@
         <v>21</v>
       </c>
       <c r="D82">
-        <f>D80*0.05</f>
+        <f>(D80*0.05)</f>
         <v>200</v>
-      </c>
-      <c r="E82">
-        <f>E81*0.05</f>
-        <v>100</v>
-      </c>
-      <c r="G82">
-        <f>G81*0.05</f>
-        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
@@ -4358,7 +4360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
         <v>7</v>
       </c>
@@ -4369,7 +4371,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
         <v>8</v>
       </c>
@@ -4380,7 +4382,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
         <v>9</v>
       </c>
@@ -4388,7 +4390,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
         <v>10</v>
       </c>
@@ -4399,7 +4401,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
         <v>44</v>
       </c>
@@ -4410,7 +4412,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>105</v>
       </c>
@@ -4421,10 +4423,13 @@
         <v>21</v>
       </c>
       <c r="D134">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2000</v>
+      </c>
+      <c r="G134">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
         <v>7</v>
       </c>
@@ -4433,10 +4438,10 @@
       </c>
       <c r="D135">
         <f>D134*0.05</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
         <v>8</v>
       </c>
@@ -4447,15 +4452,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
         <v>9</v>
       </c>
       <c r="D137">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E137">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
         <v>10</v>
       </c>
@@ -4463,10 +4471,10 @@
         <v>11</v>
       </c>
       <c r="D138">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
         <v>44</v>
       </c>
@@ -4477,7 +4485,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>106</v>
       </c>
@@ -4488,10 +4496,13 @@
         <v>21</v>
       </c>
       <c r="D140">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
+        <v>2000</v>
+      </c>
+      <c r="G140">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
         <v>7</v>
       </c>
@@ -4500,10 +4511,10 @@
       </c>
       <c r="D141">
         <f>D140*0.05</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
         <v>8</v>
       </c>
@@ -4514,15 +4525,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
         <v>9</v>
       </c>
       <c r="D143">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E143">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
         <v>10</v>
       </c>
@@ -4530,7 +4544,7 @@
         <v>11</v>
       </c>
       <c r="D144">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.2">
@@ -4678,6 +4692,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Final push with all graphs, correct parameters, and extra Word document for parameters
</commit_message>
<xml_diff>
--- a/Group Assignment MfT/input_databases/default/technologies.xlsx
+++ b/Group Assignment MfT/input_databases/default/technologies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacerato/Modelling_for_transitions_Group/Group Assignment MfT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{211B4C32-4B70-D246-8F70-E8ED390293AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{77FD70EE-D948-954A-A879-C7C67AE4104F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3560" yWindow="600" windowWidth="20540" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3535,10 +3535,10 @@
         <v>21</v>
       </c>
       <c r="D68">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="G68">
-        <v>1500</v>
+        <v>150</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="D69">
         <f>D68*0.05</f>
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -3608,10 +3608,10 @@
         <v>21</v>
       </c>
       <c r="D74">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="G74">
-        <v>1500</v>
+        <v>150</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D75">
         <f>D74*0.05</f>
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -3681,16 +3681,16 @@
         <v>21</v>
       </c>
       <c r="D80">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="E80">
-        <v>3800</v>
+        <v>1900</v>
       </c>
       <c r="F80">
-        <v>3610</v>
+        <v>1805</v>
       </c>
       <c r="G80">
-        <v>3429</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -3702,19 +3702,19 @@
       </c>
       <c r="D81">
         <f>D80*0.3</f>
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="E81">
         <f>E80*0.3</f>
-        <v>1140</v>
+        <v>570</v>
       </c>
       <c r="F81">
         <f t="shared" ref="F81:G81" si="3">F80*0.3</f>
-        <v>1083</v>
+        <v>541.5</v>
       </c>
       <c r="G81">
         <f t="shared" si="3"/>
-        <v>1028.7</v>
+        <v>514.19999999999993</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="D82">
         <f>(D80*0.05)</f>
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
@@ -4423,10 +4423,10 @@
         <v>21</v>
       </c>
       <c r="D134">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="G134">
-        <v>1500</v>
+        <v>150</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="D135">
         <f>D134*0.05</f>
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.2">
@@ -4496,10 +4496,10 @@
         <v>21</v>
       </c>
       <c r="D140">
-        <v>2000</v>
+        <v>200</v>
       </c>
       <c r="G140">
-        <v>1500</v>
+        <v>150</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.2">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="D141">
         <f>D140*0.05</f>
-        <v>100</v>
+        <v>10</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>